<commit_message>
feat(epirank): add M1/M2 metric log formatting and refresh 改 results
- add format_m1_m2_log() with stat summary, Top-N rank tables and top weighted edges to 改 and 改_Germany GUI scripts (forward + reverse)
- refresh ERA_result seqday/reverse json+xlsx for 改 (116 loops) and 改_Germany (105 loops)
</commit_message>
<xml_diff>
--- a/EpiRank_改/ERA_result_reverse_seqday_d_0.95_loops_116.xlsx
+++ b/EpiRank_改/ERA_result_reverse_seqday_d_0.95_loops_116.xlsx
@@ -1027,7 +1027,7 @@
         <v>0</v>
       </c>
       <c r="Z4" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="3" t="n">
         <v>11</v>
@@ -1636,10 +1636,10 @@
         <v>0.016941</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z8" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA8" s="3" t="n">
         <v>8</v>
@@ -1787,10 +1787,10 @@
         <v>0.009434</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA9" s="3" t="n">
         <v>2</v>
@@ -1938,10 +1938,10 @@
         <v>0.011997</v>
       </c>
       <c r="Y10" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z10" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA10" s="3" t="n">
         <v>4</v>
@@ -2558,10 +2558,10 @@
         <v>0.006602</v>
       </c>
       <c r="Y14" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z14" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA14" s="3" t="n">
         <v>6</v>
@@ -3138,10 +3138,10 @@
         <v>0.004698</v>
       </c>
       <c r="Y18" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>4</v>
@@ -3688,10 +3688,10 @@
         <v>0.009729</v>
       </c>
       <c r="Y22" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z22" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA22" s="3" t="n">
         <v>24</v>
@@ -4471,7 +4471,7 @@
         <v>0</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA28" s="3" t="n">
         <v>4</v>
@@ -5478,10 +5478,10 @@
         <v>0.01038</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA36" s="3" t="n">
         <v>0</v>
@@ -6438,10 +6438,10 @@
         <v>0.007706</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>2</v>
@@ -6798,10 +6798,10 @@
         <v>0.005831</v>
       </c>
       <c r="Y47" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z47" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA47" s="3" t="n">
         <v>0</v>
@@ -6918,10 +6918,10 @@
         <v>0.006948</v>
       </c>
       <c r="Y48" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z48" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA48" s="3" t="n">
         <v>3</v>
@@ -7881,7 +7881,7 @@
         <v>0</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA56" s="3" t="n">
         <v>2</v>
@@ -8598,7 +8598,7 @@
         <v>0.006096</v>
       </c>
       <c r="Y62" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z62" s="3" t="n">
         <v>0</v>
@@ -8958,10 +8958,10 @@
         <v>0.004618</v>
       </c>
       <c r="Y65" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z65" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA65" s="3" t="n">
         <v>6</v>
@@ -9198,10 +9198,10 @@
         <v>0.0015</v>
       </c>
       <c r="Y67" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z67" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA67" s="3" t="n">
         <v>35</v>
@@ -10758,7 +10758,7 @@
         <v>0.002616</v>
       </c>
       <c r="Y81" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z81" s="3" t="n">
         <v>0</v>
@@ -11528,7 +11528,7 @@
         <v>0.002613</v>
       </c>
       <c r="Y88" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z88" s="3" t="n">
         <v>-0</v>
@@ -11638,10 +11638,10 @@
         <v>0.003408</v>
       </c>
       <c r="Y89" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z89" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA89" s="3" t="n">
         <v>1</v>
@@ -11858,10 +11858,10 @@
         <v>0.002947</v>
       </c>
       <c r="Y91" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z91" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA91" s="3" t="n">
         <v>3</v>
@@ -11968,10 +11968,10 @@
         <v>0.003989</v>
       </c>
       <c r="Y92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA92" s="3" t="n">
         <v>1</v>
@@ -12078,10 +12078,10 @@
         <v>0.003716</v>
       </c>
       <c r="Y93" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z93" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA93" s="3" t="n">
         <v>0</v>
@@ -12738,10 +12738,10 @@
         <v>0.0059</v>
       </c>
       <c r="Y99" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z99" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA99" s="3" t="n">
         <v>0</v>
@@ -13178,10 +13178,10 @@
         <v>0.003781</v>
       </c>
       <c r="Y103" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z103" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA103" s="3" t="n">
         <v>0</v>
@@ -13398,10 +13398,10 @@
         <v>0.002789</v>
       </c>
       <c r="Y105" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z105" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA105" s="3" t="n">
         <v>1</v>
@@ -13838,10 +13838,10 @@
         <v>0.002268</v>
       </c>
       <c r="Y109" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z109" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA109" s="3" t="n">
         <v>0</v>
@@ -13951,7 +13951,7 @@
         <v>-0</v>
       </c>
       <c r="Z110" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA110" s="3" t="n">
         <v>2</v>
@@ -14058,10 +14058,10 @@
         <v>0.003672</v>
       </c>
       <c r="Y111" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z111" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA111" s="3" t="n">
         <v>0</v>
@@ -14608,10 +14608,10 @@
         <v>0.005244</v>
       </c>
       <c r="Y116" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z116" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA116" s="3" t="n">
         <v>2</v>
@@ -15268,10 +15268,10 @@
         <v>0.002014</v>
       </c>
       <c r="Y122" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z122" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA122" s="3" t="n">
         <v>3</v>
@@ -16478,10 +16478,10 @@
         <v>0.002594</v>
       </c>
       <c r="Y133" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z133" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA133" s="3" t="n">
         <v>0</v>
@@ -16698,7 +16698,7 @@
         <v>0.00191</v>
       </c>
       <c r="Y135" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z135" s="3" t="n">
         <v>-0</v>
@@ -17028,10 +17028,10 @@
         <v>0.002448</v>
       </c>
       <c r="Y138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA138" s="3" t="n">
         <v>0</v>
@@ -17138,10 +17138,10 @@
         <v>0.001759</v>
       </c>
       <c r="Y139" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z139" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA139" s="3" t="n">
         <v>1</v>
@@ -17251,7 +17251,7 @@
         <v>-0</v>
       </c>
       <c r="Z140" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA140" s="3" t="n">
         <v>3</v>
@@ -17578,7 +17578,7 @@
         <v>0.003403</v>
       </c>
       <c r="Y143" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z143" s="3" t="n">
         <v>-0</v>
@@ -17798,10 +17798,10 @@
         <v>0.002116</v>
       </c>
       <c r="Y145" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z145" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA145" s="3" t="n">
         <v>0</v>
@@ -18021,7 +18021,7 @@
         <v>-0</v>
       </c>
       <c r="Z147" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA147" s="3" t="n">
         <v>0</v>
@@ -18348,7 +18348,7 @@
         <v>0.001664</v>
       </c>
       <c r="Y150" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z150" s="3" t="n">
         <v>0</v>
@@ -18678,10 +18678,10 @@
         <v>0.002604</v>
       </c>
       <c r="Y153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>7</v>
@@ -18898,10 +18898,10 @@
         <v>0.002578</v>
       </c>
       <c r="Y155" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z155" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA155" s="3" t="n">
         <v>0</v>
@@ -19338,7 +19338,7 @@
         <v>0.002147</v>
       </c>
       <c r="Y159" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z159" s="3" t="n">
         <v>-0</v>
@@ -19558,7 +19558,7 @@
         <v>0.003002</v>
       </c>
       <c r="Y161" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z161" s="3" t="n">
         <v>-0</v>
@@ -19671,7 +19671,7 @@
         <v>-0</v>
       </c>
       <c r="Z162" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA162" s="3" t="n">
         <v>0</v>
@@ -19998,7 +19998,7 @@
         <v>0.002432</v>
       </c>
       <c r="Y165" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z165" s="3" t="n">
         <v>-0</v>
@@ -20331,7 +20331,7 @@
         <v>-0</v>
       </c>
       <c r="Z168" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA168" s="3" t="n">
         <v>2</v>
@@ -20438,10 +20438,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y169" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z169" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA169" s="3" t="n">
         <v>0</v>
@@ -20988,10 +20988,10 @@
         <v>0.001501</v>
       </c>
       <c r="Y174" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z174" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA174" s="3" t="n">
         <v>1</v>
@@ -21318,10 +21318,10 @@
         <v>0.001307</v>
       </c>
       <c r="Y177" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z177" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA177" s="3" t="n">
         <v>0</v>
@@ -21428,10 +21428,10 @@
         <v>0.002004</v>
       </c>
       <c r="Y178" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z178" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA178" s="3" t="n">
         <v>2</v>
@@ -21758,10 +21758,10 @@
         <v>0.002618</v>
       </c>
       <c r="Y181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA181" s="3" t="n">
         <v>0</v>
@@ -22641,7 +22641,7 @@
         <v>0</v>
       </c>
       <c r="Z189" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA189" s="3" t="n">
         <v>1</v>
@@ -22748,7 +22748,7 @@
         <v>0.002087</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z190" s="3" t="n">
         <v>-0</v>
@@ -23078,7 +23078,7 @@
         <v>0.002161</v>
       </c>
       <c r="Y193" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z193" s="3" t="n">
         <v>0</v>
@@ -23298,10 +23298,10 @@
         <v>0.001708</v>
       </c>
       <c r="Y195" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z195" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA195" s="3" t="n">
         <v>0</v>
@@ -23521,7 +23521,7 @@
         <v>0</v>
       </c>
       <c r="Z197" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA197" s="3" t="n">
         <v>3</v>
@@ -23628,7 +23628,7 @@
         <v>0.001192</v>
       </c>
       <c r="Y198" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z198" s="3" t="n">
         <v>0</v>
@@ -23848,10 +23848,10 @@
         <v>0.001259</v>
       </c>
       <c r="Y200" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z200" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA200" s="3" t="n">
         <v>1</v>
@@ -24068,7 +24068,7 @@
         <v>0.001326</v>
       </c>
       <c r="Y202" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z202" s="3" t="n">
         <v>-0</v>
@@ -24511,7 +24511,7 @@
         <v>0</v>
       </c>
       <c r="Z206" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA206" s="3" t="n">
         <v>3</v>
@@ -24841,7 +24841,7 @@
         <v>0</v>
       </c>
       <c r="Z209" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA209" s="3" t="n">
         <v>2</v>
@@ -24948,7 +24948,7 @@
         <v>0.002238</v>
       </c>
       <c r="Y210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
         <v>0</v>
@@ -25058,7 +25058,7 @@
         <v>0.001686</v>
       </c>
       <c r="Y211" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z211" s="3" t="n">
         <v>-0</v>
@@ -25278,10 +25278,10 @@
         <v>0.001943</v>
       </c>
       <c r="Y213" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z213" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA213" s="3" t="n">
         <v>0</v>
@@ -25501,7 +25501,7 @@
         <v>0</v>
       </c>
       <c r="Z215" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA215" s="3" t="n">
         <v>1</v>
@@ -25608,10 +25608,10 @@
         <v>0.001081</v>
       </c>
       <c r="Y216" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z216" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA216" s="3" t="n">
         <v>3</v>
@@ -26048,10 +26048,10 @@
         <v>0.00185</v>
       </c>
       <c r="Y220" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z220" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA220" s="3" t="n">
         <v>2</v>
@@ -26688,10 +26688,10 @@
         <v>0.001592</v>
       </c>
       <c r="Y226" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z226" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA226" s="3" t="n">
         <v>1</v>
@@ -26888,10 +26888,10 @@
         <v>0.00125</v>
       </c>
       <c r="Y228" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z228" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA228" s="3" t="n">
         <v>0</v>
@@ -26988,7 +26988,7 @@
         <v>0.00135</v>
       </c>
       <c r="Y229" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z229" s="3" t="n">
         <v>0</v>
@@ -27091,7 +27091,7 @@
         <v>0</v>
       </c>
       <c r="Z230" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA230" s="3" t="n">
         <v>0</v>
@@ -27188,10 +27188,10 @@
         <v>0.001237</v>
       </c>
       <c r="Y231" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z231" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA231" s="3" t="n">
         <v>5</v>
@@ -27688,7 +27688,7 @@
         <v>0.0008140000000000001</v>
       </c>
       <c r="Y236" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z236" s="3" t="n">
         <v>0</v>
@@ -27788,7 +27788,7 @@
         <v>0.001309</v>
       </c>
       <c r="Y237" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z237" s="3" t="n">
         <v>0</v>
@@ -28088,10 +28088,10 @@
         <v>0.001577</v>
       </c>
       <c r="Y240" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z240" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA240" s="3" t="n">
         <v>0</v>
@@ -28291,7 +28291,7 @@
         <v>0</v>
       </c>
       <c r="Z242" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA242" s="3" t="n">
         <v>0</v>
@@ -28388,7 +28388,7 @@
         <v>0.001556</v>
       </c>
       <c r="Y243" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z243" s="3" t="n">
         <v>-0</v>
@@ -29291,7 +29291,7 @@
         <v>0</v>
       </c>
       <c r="Z252" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA252" s="3" t="n">
         <v>0</v>
@@ -29491,7 +29491,7 @@
         <v>0</v>
       </c>
       <c r="Z254" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA254" s="3" t="n">
         <v>3</v>
@@ -29588,10 +29588,10 @@
         <v>0.000995</v>
       </c>
       <c r="Y255" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z255" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA255" s="3" t="n">
         <v>0</v>
@@ -29888,7 +29888,7 @@
         <v>0.001509</v>
       </c>
       <c r="Y258" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z258" s="3" t="n">
         <v>0</v>
@@ -30191,7 +30191,7 @@
         <v>0</v>
       </c>
       <c r="Z261" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA261" s="3" t="n">
         <v>0</v>
@@ -30288,10 +30288,10 @@
         <v>0.00143</v>
       </c>
       <c r="Y262" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z262" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA262" s="3" t="n">
         <v>0</v>
@@ -30391,7 +30391,7 @@
         <v>-0</v>
       </c>
       <c r="Z263" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA263" s="3" t="n">
         <v>1</v>
@@ -30491,7 +30491,7 @@
         <v>-0</v>
       </c>
       <c r="Z264" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA264" s="3" t="n">
         <v>0</v>
@@ -30888,7 +30888,7 @@
         <v>0.00079</v>
       </c>
       <c r="Y268" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z268" s="3" t="n">
         <v>0</v>
@@ -30988,7 +30988,7 @@
         <v>0.001019</v>
       </c>
       <c r="Y269" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z269" s="3" t="n">
         <v>-0</v>
@@ -31388,10 +31388,10 @@
         <v>0.001118</v>
       </c>
       <c r="Y273" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z273" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA273" s="3" t="n">
         <v>0</v>
@@ -31588,10 +31588,10 @@
         <v>0.001032</v>
       </c>
       <c r="Y275" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z275" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA275" s="3" t="n">
         <v>0</v>
@@ -31891,7 +31891,7 @@
         <v>-0</v>
       </c>
       <c r="Z278" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA278" s="3" t="n">
         <v>0</v>
@@ -32488,10 +32488,10 @@
         <v>0.001506</v>
       </c>
       <c r="Y284" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z284" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA284" s="3" t="n">
         <v>2</v>
@@ -32591,7 +32591,7 @@
         <v>-0</v>
       </c>
       <c r="Z285" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA285" s="3" t="n">
         <v>0</v>
@@ -32691,7 +32691,7 @@
         <v>0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>1</v>
@@ -33088,7 +33088,7 @@
         <v>0.000883</v>
       </c>
       <c r="Y290" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z290" s="3" t="n">
         <v>-0</v>
@@ -33291,7 +33291,7 @@
         <v>0</v>
       </c>
       <c r="Z292" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA292" s="3" t="n">
         <v>1</v>
@@ -33488,7 +33488,7 @@
         <v>0.0009479999999999999</v>
       </c>
       <c r="Y294" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z294" s="3" t="n">
         <v>0</v>
@@ -33688,10 +33688,10 @@
         <v>0.001087</v>
       </c>
       <c r="Y296" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z296" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA296" s="3" t="n">
         <v>9</v>
@@ -33791,7 +33791,7 @@
         <v>0</v>
       </c>
       <c r="Z297" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA297" s="3" t="n">
         <v>0</v>
@@ -34191,7 +34191,7 @@
         <v>0</v>
       </c>
       <c r="Z301" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA301" s="3" t="n">
         <v>1</v>
@@ -34291,7 +34291,7 @@
         <v>0</v>
       </c>
       <c r="Z302" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA302" s="3" t="n">
         <v>0</v>
@@ -34388,7 +34388,7 @@
         <v>0.001097</v>
       </c>
       <c r="Y303" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z303" s="3" t="n">
         <v>-0</v>
@@ -34488,7 +34488,7 @@
         <v>0.000908</v>
       </c>
       <c r="Y304" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z304" s="3" t="n">
         <v>-0</v>
@@ -34691,7 +34691,7 @@
         <v>0</v>
       </c>
       <c r="Z306" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA306" s="3" t="n">
         <v>0</v>
@@ -34888,7 +34888,7 @@
         <v>0.001184</v>
       </c>
       <c r="Y308" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z308" s="3" t="n">
         <v>0</v>
@@ -35191,7 +35191,7 @@
         <v>0</v>
       </c>
       <c r="Z311" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA311" s="3" t="n">
         <v>0</v>
@@ -35788,10 +35788,10 @@
         <v>0.001123</v>
       </c>
       <c r="Y317" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z317" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA317" s="3" t="n">
         <v>0</v>
@@ -35988,10 +35988,10 @@
         <v>0.001202</v>
       </c>
       <c r="Y319" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z319" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA319" s="3" t="n">
         <v>0</v>
@@ -36091,7 +36091,7 @@
         <v>0</v>
       </c>
       <c r="Z320" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA320" s="3" t="n">
         <v>1</v>
@@ -36488,10 +36488,10 @@
         <v>0.00087</v>
       </c>
       <c r="Y324" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z324" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA324" s="3" t="n">
         <v>0</v>
@@ -36588,7 +36588,7 @@
         <v>0.000819</v>
       </c>
       <c r="Y325" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z325" s="3" t="n">
         <v>-0</v>
@@ -37588,7 +37588,7 @@
         <v>0.000763</v>
       </c>
       <c r="Y335" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z335" s="3" t="n">
         <v>-0</v>
@@ -38288,10 +38288,10 @@
         <v>0.000725</v>
       </c>
       <c r="Y342" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z342" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA342" s="3" t="n">
         <v>1</v>
@@ -38591,7 +38591,7 @@
         <v>0</v>
       </c>
       <c r="Z345" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA345" s="3" t="n">
         <v>0</v>
@@ -38791,7 +38791,7 @@
         <v>-0</v>
       </c>
       <c r="Z347" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA347" s="3" t="n">
         <v>0</v>
@@ -39288,10 +39288,10 @@
         <v>0.000518</v>
       </c>
       <c r="Y352" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z352" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA352" s="3" t="n">
         <v>0</v>
@@ -39564,10 +39564,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.21324</v>
+        <v>0.097938</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.174906</v>
+        <v>0.128125</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.6355420000000001</v>
@@ -39626,10 +39626,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.464334</v>
+        <v>0.404628</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.428091</v>
+        <v>0.408213</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.551722</v>
@@ -40001,10 +40001,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.464334</v>
+        <v>0.404628</v>
       </c>
       <c r="E8" t="n">
-        <v>0.352584</v>
+        <v>0.312706</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40031,10 +40031,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.21324</v>
+        <v>0.097938</v>
       </c>
       <c r="E9" t="n">
-        <v>0.163438</v>
+        <v>0.069392</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40061,10 +40061,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.39334</v>
+        <v>0.376789</v>
       </c>
       <c r="E10" t="n">
-        <v>0.319962</v>
+        <v>0.305736</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40091,10 +40091,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.428091</v>
+        <v>0.408213</v>
       </c>
       <c r="E11" t="n">
-        <v>0.320074</v>
+        <v>0.311598</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40121,10 +40121,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.174906</v>
+        <v>0.128125</v>
       </c>
       <c r="E12" t="n">
-        <v>0.131345</v>
+        <v>0.094475</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40151,10 +40151,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.372746</v>
+        <v>0.359978</v>
       </c>
       <c r="E13" t="n">
-        <v>0.302824</v>
+        <v>0.291623</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>

<commit_message>
fix(epirank): compute classical Kemeny constant from full spectrum
- keep absolute spectral gap 1-|l2|/|l1| for mixing speed, compute Kemeny as sum_r 1/(1-lambda_r) with Perron root removed
- rename lambda1/lambda2 -> abs_lambda1/abs_lambda2 in transient_metrics and M1 log/panel text
- refresh ERA_result seqday/reverse json+xlsx for 改 (116 loops) and 改_Germany (105 loops)
</commit_message>
<xml_diff>
--- a/EpiRank_改/ERA_result_reverse_seqday_d_0.95_loops_116.xlsx
+++ b/EpiRank_改/ERA_result_reverse_seqday_d_0.95_loops_116.xlsx
@@ -1179,10 +1179,10 @@
         <v>0.01205</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="3" t="n">
         <v>11</v>
@@ -1334,10 +1334,10 @@
         <v>0.006652</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA6" s="3" t="n">
         <v>11</v>
@@ -1636,10 +1636,10 @@
         <v>0.016941</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="3" t="n">
         <v>8</v>
@@ -1787,10 +1787,10 @@
         <v>0.009434</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z9" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA9" s="3" t="n">
         <v>2</v>
@@ -1938,7 +1938,7 @@
         <v>0.011997</v>
       </c>
       <c r="Y10" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="3" t="n">
         <v>-0</v>
@@ -2708,10 +2708,10 @@
         <v>0.008586</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z15" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA15" s="3" t="n">
         <v>3</v>
@@ -2858,10 +2858,10 @@
         <v>0.008274999999999999</v>
       </c>
       <c r="Y16" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA16" s="3" t="n">
         <v>4</v>
@@ -3138,10 +3138,10 @@
         <v>0.004698</v>
       </c>
       <c r="Y18" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>4</v>
@@ -3278,10 +3278,10 @@
         <v>0.011024</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="3" t="n">
         <v>8</v>
@@ -3948,10 +3948,10 @@
         <v>0.007023</v>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z24" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA24" s="3" t="n">
         <v>8</v>
@@ -4598,10 +4598,10 @@
         <v>0.004713</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA29" s="3" t="n">
         <v>7</v>
@@ -4988,10 +4988,10 @@
         <v>0.008265</v>
       </c>
       <c r="Y32" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z32" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA32" s="3" t="n">
         <v>5</v>
@@ -5478,10 +5478,10 @@
         <v>0.01038</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA36" s="3" t="n">
         <v>0</v>
@@ -6318,10 +6318,10 @@
         <v>0.004917</v>
       </c>
       <c r="Y43" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z43" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA43" s="3" t="n">
         <v>2</v>
@@ -6558,10 +6558,10 @@
         <v>0.006149</v>
       </c>
       <c r="Y45" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z45" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA45" s="3" t="n">
         <v>5</v>
@@ -6918,10 +6918,10 @@
         <v>0.006948</v>
       </c>
       <c r="Y48" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z48" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA48" s="3" t="n">
         <v>3</v>
@@ -7881,7 +7881,7 @@
         <v>0</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA56" s="3" t="n">
         <v>2</v>
@@ -8598,10 +8598,10 @@
         <v>0.006096</v>
       </c>
       <c r="Y62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z62" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA62" s="3" t="n">
         <v>1</v>
@@ -9198,10 +9198,10 @@
         <v>0.0015</v>
       </c>
       <c r="Y67" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z67" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA67" s="3" t="n">
         <v>35</v>
@@ -9548,7 +9548,7 @@
         <v>0.002648</v>
       </c>
       <c r="Y70" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z70" s="3" t="n">
         <v>0</v>
@@ -10208,7 +10208,7 @@
         <v>0.002491</v>
       </c>
       <c r="Y76" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z76" s="3" t="n">
         <v>0</v>
@@ -10758,7 +10758,7 @@
         <v>0.002616</v>
       </c>
       <c r="Y81" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z81" s="3" t="n">
         <v>0</v>
@@ -11531,7 +11531,7 @@
         <v>0</v>
       </c>
       <c r="Z88" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA88" s="3" t="n">
         <v>2</v>
@@ -11971,7 +11971,7 @@
         <v>-0</v>
       </c>
       <c r="Z92" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA92" s="3" t="n">
         <v>1</v>
@@ -12628,10 +12628,10 @@
         <v>0.003197</v>
       </c>
       <c r="Y98" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z98" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA98" s="3" t="n">
         <v>1</v>
@@ -12738,10 +12738,10 @@
         <v>0.0059</v>
       </c>
       <c r="Y99" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z99" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA99" s="3" t="n">
         <v>0</v>
@@ -13178,10 +13178,10 @@
         <v>0.003781</v>
       </c>
       <c r="Y103" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z103" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA103" s="3" t="n">
         <v>0</v>
@@ -13508,10 +13508,10 @@
         <v>0.003882</v>
       </c>
       <c r="Y106" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z106" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA106" s="3" t="n">
         <v>0</v>
@@ -13948,7 +13948,7 @@
         <v>0.001988</v>
       </c>
       <c r="Y110" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z110" s="3" t="n">
         <v>0</v>
@@ -14388,10 +14388,10 @@
         <v>0.002802</v>
       </c>
       <c r="Y114" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z114" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA114" s="3" t="n">
         <v>0</v>
@@ -14498,10 +14498,10 @@
         <v>0.002806</v>
       </c>
       <c r="Y115" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z115" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA115" s="3" t="n">
         <v>0</v>
@@ -14608,10 +14608,10 @@
         <v>0.005244</v>
       </c>
       <c r="Y116" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z116" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA116" s="3" t="n">
         <v>2</v>
@@ -14718,7 +14718,7 @@
         <v>0.004473</v>
       </c>
       <c r="Y117" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z117" s="3" t="n">
         <v>0</v>
@@ -14938,10 +14938,10 @@
         <v>0.002833</v>
       </c>
       <c r="Y119" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z119" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA119" s="3" t="n">
         <v>0</v>
@@ -15048,10 +15048,10 @@
         <v>0.002833</v>
       </c>
       <c r="Y120" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z120" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA120" s="3" t="n">
         <v>1</v>
@@ -15268,10 +15268,10 @@
         <v>0.002014</v>
       </c>
       <c r="Y122" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z122" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA122" s="3" t="n">
         <v>3</v>
@@ -15378,10 +15378,10 @@
         <v>0.004587</v>
       </c>
       <c r="Y123" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z123" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA123" s="3" t="n">
         <v>0</v>
@@ -15488,10 +15488,10 @@
         <v>0.003344</v>
       </c>
       <c r="Y124" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>3</v>
@@ -15601,7 +15601,7 @@
         <v>0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>2</v>
@@ -15711,7 +15711,7 @@
         <v>0</v>
       </c>
       <c r="Z126" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA126" s="3" t="n">
         <v>0</v>
@@ -16148,10 +16148,10 @@
         <v>0.002496</v>
       </c>
       <c r="Y130" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z130" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA130" s="3" t="n">
         <v>1</v>
@@ -17028,7 +17028,7 @@
         <v>0.002448</v>
       </c>
       <c r="Y138" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z138" s="3" t="n">
         <v>0</v>
@@ -17138,7 +17138,7 @@
         <v>0.001759</v>
       </c>
       <c r="Y139" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z139" s="3" t="n">
         <v>0</v>
@@ -17248,10 +17248,10 @@
         <v>0.002964</v>
       </c>
       <c r="Y140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z140" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z140" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA140" s="3" t="n">
         <v>3</v>
@@ -17358,10 +17358,10 @@
         <v>0.00302</v>
       </c>
       <c r="Y141" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z141" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA141" s="3" t="n">
         <v>5</v>
@@ -17578,10 +17578,10 @@
         <v>0.003403</v>
       </c>
       <c r="Y143" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z143" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA143" s="3" t="n">
         <v>0</v>
@@ -18348,10 +18348,10 @@
         <v>0.001664</v>
       </c>
       <c r="Y150" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z150" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA150" s="3" t="n">
         <v>0</v>
@@ -18461,7 +18461,7 @@
         <v>-0</v>
       </c>
       <c r="Z151" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA151" s="3" t="n">
         <v>1</v>
@@ -18678,10 +18678,10 @@
         <v>0.002604</v>
       </c>
       <c r="Y153" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>7</v>
@@ -19118,10 +19118,10 @@
         <v>0.001714</v>
       </c>
       <c r="Y157" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z157" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA157" s="3" t="n">
         <v>2</v>
@@ -19341,7 +19341,7 @@
         <v>0</v>
       </c>
       <c r="Z159" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA159" s="3" t="n">
         <v>1</v>
@@ -19561,7 +19561,7 @@
         <v>-0</v>
       </c>
       <c r="Z161" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA161" s="3" t="n">
         <v>0</v>
@@ -19668,7 +19668,7 @@
         <v>0.003364</v>
       </c>
       <c r="Y162" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z162" s="3" t="n">
         <v>0</v>
@@ -19778,10 +19778,10 @@
         <v>0.002174</v>
       </c>
       <c r="Y163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA163" s="3" t="n">
         <v>1</v>
@@ -19998,10 +19998,10 @@
         <v>0.002432</v>
       </c>
       <c r="Y165" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z165" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA165" s="3" t="n">
         <v>1</v>
@@ -20328,7 +20328,7 @@
         <v>0.001621</v>
       </c>
       <c r="Y168" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z168" s="3" t="n">
         <v>0</v>
@@ -20438,10 +20438,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y169" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z169" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA169" s="3" t="n">
         <v>0</v>
@@ -20658,10 +20658,10 @@
         <v>0.001901</v>
       </c>
       <c r="Y171" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z171" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA171" s="3" t="n">
         <v>0</v>
@@ -21098,10 +21098,10 @@
         <v>0.001399</v>
       </c>
       <c r="Y175" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z175" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA175" s="3" t="n">
         <v>1</v>
@@ -21208,10 +21208,10 @@
         <v>0.002542</v>
       </c>
       <c r="Y176" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>1</v>
@@ -21318,7 +21318,7 @@
         <v>0.001307</v>
       </c>
       <c r="Y177" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z177" s="3" t="n">
         <v>-0</v>
@@ -21431,7 +21431,7 @@
         <v>-0</v>
       </c>
       <c r="Z178" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA178" s="3" t="n">
         <v>2</v>
@@ -21758,10 +21758,10 @@
         <v>0.002618</v>
       </c>
       <c r="Y181" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z181" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA181" s="3" t="n">
         <v>0</v>
@@ -22198,10 +22198,10 @@
         <v>0.001235</v>
       </c>
       <c r="Y185" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z185" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA185" s="3" t="n">
         <v>1</v>
@@ -22421,7 +22421,7 @@
         <v>0</v>
       </c>
       <c r="Z187" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA187" s="3" t="n">
         <v>0</v>
@@ -22641,7 +22641,7 @@
         <v>0</v>
       </c>
       <c r="Z189" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA189" s="3" t="n">
         <v>1</v>
@@ -22748,10 +22748,10 @@
         <v>0.002087</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA190" s="3" t="n">
         <v>0</v>
@@ -22858,10 +22858,10 @@
         <v>0.001644</v>
       </c>
       <c r="Y191" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z191" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA191" s="3" t="n">
         <v>1</v>
@@ -23298,10 +23298,10 @@
         <v>0.001708</v>
       </c>
       <c r="Y195" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z195" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA195" s="3" t="n">
         <v>0</v>
@@ -23411,7 +23411,7 @@
         <v>0</v>
       </c>
       <c r="Z196" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA196" s="3" t="n">
         <v>1</v>
@@ -23518,10 +23518,10 @@
         <v>0.0009700000000000001</v>
       </c>
       <c r="Y197" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z197" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA197" s="3" t="n">
         <v>3</v>
@@ -23628,10 +23628,10 @@
         <v>0.001192</v>
       </c>
       <c r="Y198" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z198" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z198" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA198" s="3" t="n">
         <v>0</v>
@@ -23738,10 +23738,10 @@
         <v>0.001669</v>
       </c>
       <c r="Y199" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z199" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA199" s="3" t="n">
         <v>0</v>
@@ -24068,10 +24068,10 @@
         <v>0.001326</v>
       </c>
       <c r="Y202" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z202" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA202" s="3" t="n">
         <v>0</v>
@@ -24511,7 +24511,7 @@
         <v>0</v>
       </c>
       <c r="Z206" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA206" s="3" t="n">
         <v>3</v>
@@ -24838,10 +24838,10 @@
         <v>0.001782</v>
       </c>
       <c r="Y209" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z209" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA209" s="3" t="n">
         <v>2</v>
@@ -25168,7 +25168,7 @@
         <v>0.002084</v>
       </c>
       <c r="Y212" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z212" s="3" t="n">
         <v>0</v>
@@ -25278,10 +25278,10 @@
         <v>0.001943</v>
       </c>
       <c r="Y213" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z213" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA213" s="3" t="n">
         <v>0</v>
@@ -25388,10 +25388,10 @@
         <v>0.001245</v>
       </c>
       <c r="Y214" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z214" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA214" s="3" t="n">
         <v>0</v>
@@ -25611,7 +25611,7 @@
         <v>-0</v>
       </c>
       <c r="Z216" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA216" s="3" t="n">
         <v>3</v>
@@ -25938,10 +25938,10 @@
         <v>0.00315</v>
       </c>
       <c r="Y219" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z219" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA219" s="3" t="n">
         <v>0</v>
@@ -26048,10 +26048,10 @@
         <v>0.00185</v>
       </c>
       <c r="Y220" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z220" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA220" s="3" t="n">
         <v>2</v>
@@ -26271,7 +26271,7 @@
         <v>0</v>
       </c>
       <c r="Z222" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA222" s="3" t="n">
         <v>3</v>
@@ -26488,7 +26488,7 @@
         <v>0.00209</v>
       </c>
       <c r="Y224" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z224" s="3" t="n">
         <v>0</v>
@@ -26688,7 +26688,7 @@
         <v>0.001592</v>
       </c>
       <c r="Y226" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z226" s="3" t="n">
         <v>0</v>
@@ -26888,7 +26888,7 @@
         <v>0.00125</v>
       </c>
       <c r="Y228" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z228" s="3" t="n">
         <v>0</v>
@@ -26988,7 +26988,7 @@
         <v>0.00135</v>
       </c>
       <c r="Y229" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z229" s="3" t="n">
         <v>0</v>
@@ -27091,7 +27091,7 @@
         <v>0</v>
       </c>
       <c r="Z230" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA230" s="3" t="n">
         <v>0</v>
@@ -27191,7 +27191,7 @@
         <v>-0</v>
       </c>
       <c r="Z231" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA231" s="3" t="n">
         <v>5</v>
@@ -27388,10 +27388,10 @@
         <v>0.002059</v>
       </c>
       <c r="Y233" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z233" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA233" s="3" t="n">
         <v>0</v>
@@ -27688,7 +27688,7 @@
         <v>0.0008140000000000001</v>
       </c>
       <c r="Y236" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z236" s="3" t="n">
         <v>0</v>
@@ -27788,7 +27788,7 @@
         <v>0.001309</v>
       </c>
       <c r="Y237" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z237" s="3" t="n">
         <v>0</v>
@@ -28188,10 +28188,10 @@
         <v>0.001152</v>
       </c>
       <c r="Y241" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z241" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA241" s="3" t="n">
         <v>0</v>
@@ -28288,7 +28288,7 @@
         <v>0.001386</v>
       </c>
       <c r="Y242" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z242" s="3" t="n">
         <v>-0</v>
@@ -28388,10 +28388,10 @@
         <v>0.001556</v>
       </c>
       <c r="Y243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA243" s="3" t="n">
         <v>0</v>
@@ -28688,10 +28688,10 @@
         <v>0.001119</v>
       </c>
       <c r="Y246" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z246" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA246" s="3" t="n">
         <v>6</v>
@@ -28888,10 +28888,10 @@
         <v>0.000905</v>
       </c>
       <c r="Y248" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z248" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA248" s="3" t="n">
         <v>0</v>
@@ -28988,10 +28988,10 @@
         <v>0.001255</v>
       </c>
       <c r="Y249" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z249" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA249" s="3" t="n">
         <v>0</v>
@@ -29191,7 +29191,7 @@
         <v>0</v>
       </c>
       <c r="Z251" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA251" s="3" t="n">
         <v>0</v>
@@ -29291,7 +29291,7 @@
         <v>0</v>
       </c>
       <c r="Z252" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA252" s="3" t="n">
         <v>0</v>
@@ -29388,7 +29388,7 @@
         <v>0.00164</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z253" s="3" t="n">
         <v>-0</v>
@@ -29491,7 +29491,7 @@
         <v>0</v>
       </c>
       <c r="Z254" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA254" s="3" t="n">
         <v>3</v>
@@ -29588,7 +29588,7 @@
         <v>0.000995</v>
       </c>
       <c r="Y255" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z255" s="3" t="n">
         <v>-0</v>
@@ -29788,10 +29788,10 @@
         <v>0.001036</v>
       </c>
       <c r="Y257" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z257" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA257" s="3" t="n">
         <v>2</v>
@@ -30088,10 +30088,10 @@
         <v>0.001877</v>
       </c>
       <c r="Y260" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z260" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA260" s="3" t="n">
         <v>0</v>
@@ -30188,7 +30188,7 @@
         <v>0.000867</v>
       </c>
       <c r="Y261" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z261" s="3" t="n">
         <v>-0</v>
@@ -30288,7 +30288,7 @@
         <v>0.00143</v>
       </c>
       <c r="Y262" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z262" s="3" t="n">
         <v>-0</v>
@@ -30388,7 +30388,7 @@
         <v>0.001296</v>
       </c>
       <c r="Y263" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z263" s="3" t="n">
         <v>0</v>
@@ -30491,7 +30491,7 @@
         <v>-0</v>
       </c>
       <c r="Z264" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA264" s="3" t="n">
         <v>0</v>
@@ -30888,10 +30888,10 @@
         <v>0.00079</v>
       </c>
       <c r="Y268" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z268" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z268" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA268" s="3" t="n">
         <v>1</v>
@@ -30988,10 +30988,10 @@
         <v>0.001019</v>
       </c>
       <c r="Y269" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z269" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA269" s="3" t="n">
         <v>0</v>
@@ -31088,10 +31088,10 @@
         <v>0.001378</v>
       </c>
       <c r="Y270" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z270" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA270" s="3" t="n">
         <v>2</v>
@@ -31188,7 +31188,7 @@
         <v>0.001352</v>
       </c>
       <c r="Y271" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z271" s="3" t="n">
         <v>-0</v>
@@ -31391,7 +31391,7 @@
         <v>-0</v>
       </c>
       <c r="Z273" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA273" s="3" t="n">
         <v>0</v>
@@ -31588,10 +31588,10 @@
         <v>0.001032</v>
       </c>
       <c r="Y275" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z275" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA275" s="3" t="n">
         <v>0</v>
@@ -31688,10 +31688,10 @@
         <v>0.001773</v>
       </c>
       <c r="Y276" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z276" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA276" s="3" t="n">
         <v>1</v>
@@ -31791,7 +31791,7 @@
         <v>0</v>
       </c>
       <c r="Z277" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA277" s="3" t="n">
         <v>2</v>
@@ -31888,7 +31888,7 @@
         <v>0.000785</v>
       </c>
       <c r="Y278" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z278" s="3" t="n">
         <v>0</v>
@@ -32388,10 +32388,10 @@
         <v>0.00126</v>
       </c>
       <c r="Y283" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z283" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA283" s="3" t="n">
         <v>0</v>
@@ -32591,7 +32591,7 @@
         <v>-0</v>
       </c>
       <c r="Z285" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA285" s="3" t="n">
         <v>0</v>
@@ -33491,7 +33491,7 @@
         <v>-0</v>
       </c>
       <c r="Z294" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA294" s="3" t="n">
         <v>0</v>
@@ -33791,7 +33791,7 @@
         <v>0</v>
       </c>
       <c r="Z297" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA297" s="3" t="n">
         <v>0</v>
@@ -33888,7 +33888,7 @@
         <v>0.00108</v>
       </c>
       <c r="Y298" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z298" s="3" t="n">
         <v>0</v>
@@ -34488,10 +34488,10 @@
         <v>0.000908</v>
       </c>
       <c r="Y304" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z304" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA304" s="3" t="n">
         <v>0</v>
@@ -34891,7 +34891,7 @@
         <v>-0</v>
       </c>
       <c r="Z308" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA308" s="3" t="n">
         <v>0</v>
@@ -35288,10 +35288,10 @@
         <v>0.000773</v>
       </c>
       <c r="Y312" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z312" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA312" s="3" t="n">
         <v>0</v>
@@ -35488,7 +35488,7 @@
         <v>0.000827</v>
       </c>
       <c r="Y314" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z314" s="3" t="n">
         <v>-0</v>
@@ -35688,10 +35688,10 @@
         <v>0.000803</v>
       </c>
       <c r="Y316" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z316" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA316" s="3" t="n">
         <v>1</v>
@@ -35988,7 +35988,7 @@
         <v>0.001202</v>
       </c>
       <c r="Y319" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z319" s="3" t="n">
         <v>-0</v>
@@ -36091,7 +36091,7 @@
         <v>0</v>
       </c>
       <c r="Z320" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA320" s="3" t="n">
         <v>1</v>
@@ -36488,10 +36488,10 @@
         <v>0.00087</v>
       </c>
       <c r="Y324" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z324" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA324" s="3" t="n">
         <v>0</v>
@@ -36591,7 +36591,7 @@
         <v>0</v>
       </c>
       <c r="Z325" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA325" s="3" t="n">
         <v>3</v>
@@ -36891,7 +36891,7 @@
         <v>0</v>
       </c>
       <c r="Z328" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA328" s="3" t="n">
         <v>0</v>
@@ -36991,7 +36991,7 @@
         <v>0</v>
       </c>
       <c r="Z329" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA329" s="3" t="n">
         <v>0</v>
@@ -37591,7 +37591,7 @@
         <v>0</v>
       </c>
       <c r="Z335" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA335" s="3" t="n">
         <v>0</v>
@@ -37688,7 +37688,7 @@
         <v>0.001203</v>
       </c>
       <c r="Y336" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z336" s="3" t="n">
         <v>-0</v>
@@ -38591,7 +38591,7 @@
         <v>0</v>
       </c>
       <c r="Z345" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA345" s="3" t="n">
         <v>0</v>
@@ -38788,10 +38788,10 @@
         <v>0.000592</v>
       </c>
       <c r="Y347" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z347" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA347" s="3" t="n">
         <v>0</v>
@@ -39288,10 +39288,10 @@
         <v>0.000518</v>
       </c>
       <c r="Y352" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z352" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA352" s="3" t="n">
         <v>0</v>
@@ -39564,10 +39564,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.097938</v>
+        <v>0.121384</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.128125</v>
+        <v>0.10078</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.6355420000000001</v>
@@ -39626,10 +39626,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.404628</v>
+        <v>0.363999</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.408213</v>
+        <v>0.370114</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.551722</v>
@@ -40001,10 +40001,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.404628</v>
+        <v>0.363999</v>
       </c>
       <c r="E8" t="n">
-        <v>0.312706</v>
+        <v>0.278623</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40031,10 +40031,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.097938</v>
+        <v>0.121384</v>
       </c>
       <c r="E9" t="n">
-        <v>0.069392</v>
+        <v>0.08966499999999999</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40061,10 +40061,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.376789</v>
+        <v>0.329255</v>
       </c>
       <c r="E10" t="n">
-        <v>0.305736</v>
+        <v>0.266812</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40091,10 +40091,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.408213</v>
+        <v>0.370114</v>
       </c>
       <c r="E11" t="n">
-        <v>0.311598</v>
+        <v>0.278873</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40121,10 +40121,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.128125</v>
+        <v>0.10078</v>
       </c>
       <c r="E12" t="n">
-        <v>0.094475</v>
+        <v>0.07451199999999999</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40151,10 +40151,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.359978</v>
+        <v>0.329593</v>
       </c>
       <c r="E13" t="n">
-        <v>0.291623</v>
+        <v>0.267596</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>